<commit_message>
Match case table template to the reference screenshot
Use measured column widths, row heights, colors and zebra rows; keep
three empty rows and move the fill-in notes to a separate sheet.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VjhVaCQqFPyHRJT8AcSn8J
</commit_message>
<xml_diff>
--- a/cases_template.xlsx
+++ b/cases_template.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Кейсы" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Памятка" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -52,9 +53,6 @@
     <t xml:space="preserve">Reg2Dep, %</t>
   </si>
   <si>
-    <t xml:space="preserve">Итого</t>
-  </si>
-  <si>
     <t xml:space="preserve">Как заполнять</t>
   </si>
   <si>
@@ -64,10 +62,13 @@
     <t xml:space="preserve">CPA (FTD) здесь — число первых депозитов (штуки), а не цена одного депозита.</t>
   </si>
   <si>
-    <t xml:space="preserve">Синие столбцы считаются сами, их не меняют: Доход = Спенд + Профит · ROI = Профит ÷ Спенд · Click2Reg = Регистрации ÷ Клики · Reg2Dep = CPA (FTD) ÷ Регистрации.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROI считается от профита (не доход ÷ спенд). Пока поля не заполнены, расчётные ячейки пустые. Спенд и профит — в долларах, числом без знака $.</t>
+    <t xml:space="preserve">Синие столбцы и ROI считаются сами, их не меняют: Доход = Спенд + Профит · ROI = Профит ÷ Спенд · Click2Reg = Регистрации ÷ Клики · Reg2Dep = CPA (FTD) ÷ Регистрации.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROI считается от профита (не доход ÷ спенд). Пока поля пусты, расчётные ячейки пустые. Спенд и профит — в долларах, числом без знака $.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Чтобы добавить строку: выделите последнюю строку таблицы и протяните вниз за правый нижний угол.</t>
   </si>
 </sst>
 </file>
@@ -79,7 +80,7 @@
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0\ %"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -104,59 +105,51 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFF5D86E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFF5D86E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9FC7F3"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FFF2F2F2"/>
+      <color rgb="FFC9CAD1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFD966"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFD966"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF8DB8F2"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFF2F2F2"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF9A9BA3"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -165,14 +158,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF26272E"/>
-        <bgColor rgb="FF1B1C21"/>
+        <fgColor rgb="FF1F1E24"/>
+        <bgColor rgb="FF201F25"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B1C21"/>
-        <bgColor rgb="FF26272E"/>
+        <fgColor rgb="FF1A191F"/>
+        <bgColor rgb="FF1F1E24"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF205C3C"/>
+        <bgColor rgb="FF3B3A41"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF201F25"/>
+        <bgColor rgb="FF1F1E24"/>
       </patternFill>
     </fill>
   </fills>
@@ -186,16 +191,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FF3A3B44"/>
+        <color rgb="FF3B3A41"/>
       </left>
       <right style="thin">
-        <color rgb="FF3A3B44"/>
+        <color rgb="FF3B3A41"/>
       </right>
       <top style="thin">
-        <color rgb="FF3A3B44"/>
+        <color rgb="FF3B3A41"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF3A3B44"/>
+        <color rgb="FF3B3A41"/>
       </bottom>
       <diagonal/>
     </border>
@@ -225,7 +230,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -250,7 +255,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -258,19 +263,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -283,15 +300,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF1E6B3A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -303,16 +311,16 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF1E6B3A"/>
+      <rgbColor rgb="FF205C3C"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFC9CAD1"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -330,10 +338,10 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF8DB8F2"/>
+      <rgbColor rgb="FF9FC7F3"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFD966"/>
+      <rgbColor rgb="FFF5D86E"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -341,15 +349,15 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF9A9BA3"/>
-      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF1A191F"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF1B1C21"/>
-      <rgbColor rgb="FF26272E"/>
+      <rgbColor rgb="FF1F1E24"/>
+      <rgbColor rgb="FF201F25"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF3A3B44"/>
+      <rgbColor rgb="FF3B3A41"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -533,22 +541,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1E6B3A"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="19.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17.57"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -580,7 +588,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
       <c r="B2" s="3"/>
       <c r="C2" s="4"/>
@@ -604,11 +612,11 @@
         <v/>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5" t="str">
+    <row r="3" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11" t="str">
         <f aca="false">IF(AND(ISNUMBER(B3),ISNUMBER(C3)),B3+C3,"")</f>
         <v/>
       </c>
@@ -616,19 +624,19 @@
         <f aca="false">IF(AND(ISNUMBER(B3),ISNUMBER(C3),B3&gt;0),C3/B3,"")</f>
         <v/>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="7" t="str">
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="12" t="str">
         <f aca="false">IF(AND(ISNUMBER(F3),ISNUMBER(G3),F3&gt;0),G3/F3,"")</f>
         <v/>
       </c>
-      <c r="J3" s="7" t="str">
+      <c r="J3" s="12" t="str">
         <f aca="false">IF(AND(ISNUMBER(G3),ISNUMBER(H3),G3&gt;0),H3/G3,"")</f>
         <v/>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
       <c r="B4" s="3"/>
       <c r="C4" s="4"/>
@@ -652,202 +660,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B5),ISNUMBER(C5)),B5+C5,"")</f>
-        <v/>
-      </c>
-      <c r="E5" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B5),ISNUMBER(C5),B5&gt;0),C5/B5,"")</f>
-        <v/>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="7" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F5),ISNUMBER(G5),F5&gt;0),G5/F5,"")</f>
-        <v/>
-      </c>
-      <c r="J5" s="7" t="str">
-        <f aca="false">IF(AND(ISNUMBER(G5),ISNUMBER(H5),G5&gt;0),H5/G5,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B6),ISNUMBER(C6)),B6+C6,"")</f>
-        <v/>
-      </c>
-      <c r="E6" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B6),ISNUMBER(C6),B6&gt;0),C6/B6,"")</f>
-        <v/>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="7" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F6),ISNUMBER(G6),F6&gt;0),G6/F6,"")</f>
-        <v/>
-      </c>
-      <c r="J6" s="7" t="str">
-        <f aca="false">IF(AND(ISNUMBER(G6),ISNUMBER(H6),G6&gt;0),H6/G6,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B7),ISNUMBER(C7)),B7+C7,"")</f>
-        <v/>
-      </c>
-      <c r="E7" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B7),ISNUMBER(C7),B7&gt;0),C7/B7,"")</f>
-        <v/>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="7" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F7),ISNUMBER(G7),F7&gt;0),G7/F7,"")</f>
-        <v/>
-      </c>
-      <c r="J7" s="7" t="str">
-        <f aca="false">IF(AND(ISNUMBER(G7),ISNUMBER(H7),G7&gt;0),H7/G7,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="8" t="str">
-        <f aca="false">IF(COUNT(B2:B7)=0,"",SUM(B2:B7))</f>
-        <v/>
-      </c>
-      <c r="C8" s="8" t="str">
-        <f aca="false">IF(COUNT(C2:C7)=0,"",SUM(C2:C7))</f>
-        <v/>
-      </c>
-      <c r="D8" s="8" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B8),ISNUMBER(C8)),B8+C8,"")</f>
-        <v/>
-      </c>
-      <c r="E8" s="9" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B8),ISNUMBER(C8),B8&gt;0),C8/B8,"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="8" t="str">
-        <f aca="false">IF(COUNT(F2:F7)=0,"",SUM(F2:F7))</f>
-        <v/>
-      </c>
-      <c r="G8" s="8" t="str">
-        <f aca="false">IF(COUNT(G2:G7)=0,"",SUM(G2:G7))</f>
-        <v/>
-      </c>
-      <c r="H8" s="8" t="str">
-        <f aca="false">IF(COUNT(H2:H7)=0,"",SUM(H2:H7))</f>
-        <v/>
-      </c>
-      <c r="I8" s="9" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F8),ISNUMBER(G8),F8&gt;0),G8/F8,"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="9" t="str">
-        <f aca="false">IF(AND(ISNUMBER(G8),ISNUMBER(H8),G8&gt;0),H8/G8,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-    </row>
-    <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-    </row>
-    <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-    </row>
-    <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A14:J14"/>
-  </mergeCells>
-  <conditionalFormatting sqref="E2:E8">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>ISNUMBER(E2)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -856,4 +669,56 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>